<commit_message>
fix(pricing): enforce strict +/-10% max change after rounding, calculate 12-week current price, 2-year horizon metrics, and 18 unit tests
</commit_message>
<xml_diff>
--- a/outputs/pricing/pricing_optimization.xlsx
+++ b/outputs/pricing/pricing_optimization.xlsx
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1829983.55</v>
+        <v>1811967.34</v>
       </c>
     </row>
     <row r="5">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1952996.32</v>
+        <v>1914692.33</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123012.77</v>
+        <v>102724.99</v>
       </c>
     </row>
     <row r="7">
@@ -488,7 +488,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6.72 %</t>
+          <t>5.67 %</t>
         </is>
       </c>
     </row>
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -678,37 +678,37 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>3.008173076923077</v>
+        <v>3.24</v>
       </c>
       <c r="K2" t="n">
-        <v>6.016346153846154</v>
+        <v>6.49</v>
       </c>
       <c r="L2" t="n">
-        <v>5.49</v>
+        <v>5.99</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.08749999999999999</v>
+        <v>-0.077</v>
       </c>
       <c r="N2" t="n">
         <v>11370</v>
       </c>
       <c r="O2" t="n">
-        <v>15750.55</v>
+        <v>15125.22</v>
       </c>
       <c r="P2" t="n">
-        <v>68405.85576923077</v>
+        <v>73791.3</v>
       </c>
       <c r="Q2" t="n">
-        <v>86470.53999999999</v>
+        <v>90600.06</v>
       </c>
       <c r="R2" t="n">
-        <v>34202.92788461538</v>
+        <v>36952.5</v>
       </c>
       <c r="S2" t="n">
-        <v>39090.15</v>
+        <v>41594.35</v>
       </c>
       <c r="T2" t="n">
-        <v>4887.22</v>
+        <v>4641.85</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -751,37 +751,37 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>3.907912621359223</v>
+        <v>4.12</v>
       </c>
       <c r="K3" t="n">
-        <v>7.815825242718446</v>
+        <v>8.25</v>
       </c>
       <c r="L3" t="n">
         <v>7.49</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.0417</v>
+        <v>-0.0921</v>
       </c>
       <c r="N3" t="n">
         <v>9974</v>
       </c>
       <c r="O3" t="n">
-        <v>12290.73</v>
+        <v>16022.96</v>
       </c>
       <c r="P3" t="n">
-        <v>77955.04097087379</v>
+        <v>82285.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>92057.56</v>
+        <v>120011.95</v>
       </c>
       <c r="R3" t="n">
-        <v>38977.52048543689</v>
+        <v>41192.62</v>
       </c>
       <c r="S3" t="n">
-        <v>44026.46</v>
+        <v>53997.36</v>
       </c>
       <c r="T3" t="n">
-        <v>5048.94</v>
+        <v>12804.74</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -824,37 +824,37 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.8373076923076923</v>
+        <v>0.82</v>
       </c>
       <c r="K4" t="n">
-        <v>1.674615384615385</v>
+        <v>1.65</v>
       </c>
       <c r="L4" t="n">
-        <v>1.99</v>
+        <v>1.49</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1883</v>
+        <v>-0.097</v>
       </c>
       <c r="N4" t="n">
         <v>40942</v>
       </c>
       <c r="O4" t="n">
-        <v>29867.4</v>
+        <v>49332.87</v>
       </c>
       <c r="P4" t="n">
-        <v>68562.10307692307</v>
+        <v>67554.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>59436.12</v>
+        <v>73505.97</v>
       </c>
       <c r="R4" t="n">
-        <v>34281.05153846154</v>
+        <v>33981.86</v>
       </c>
       <c r="S4" t="n">
-        <v>34427.92</v>
+        <v>33053.02</v>
       </c>
       <c r="T4" t="n">
-        <v>146.87</v>
+        <v>-928.84</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -897,37 +897,37 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.855576923076923</v>
+        <v>0.82</v>
       </c>
       <c r="K5" t="n">
-        <v>1.711153846153846</v>
+        <v>1.65</v>
       </c>
       <c r="L5" t="n">
-        <v>1.99</v>
+        <v>1.49</v>
       </c>
       <c r="M5" t="n">
-        <v>0.163</v>
+        <v>-0.097</v>
       </c>
       <c r="N5" t="n">
         <v>27126</v>
       </c>
       <c r="O5" t="n">
-        <v>21311.52</v>
+        <v>31928.13</v>
       </c>
       <c r="P5" t="n">
-        <v>46416.75923076922</v>
+        <v>44757.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>42409.93</v>
+        <v>47572.91</v>
       </c>
       <c r="R5" t="n">
-        <v>23208.37961538461</v>
+        <v>22514.58</v>
       </c>
       <c r="S5" t="n">
-        <v>24176.28</v>
+        <v>21391.85</v>
       </c>
       <c r="T5" t="n">
-        <v>967.9</v>
+        <v>-1122.73</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -970,37 +970,37 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1.852727272727273</v>
+        <v>1.88</v>
       </c>
       <c r="K6" t="n">
-        <v>3.705454545454545</v>
+        <v>3.75</v>
       </c>
       <c r="L6" t="n">
         <v>3.49</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.0581</v>
+        <v>-0.0693</v>
       </c>
       <c r="N6" t="n">
         <v>19954</v>
       </c>
       <c r="O6" t="n">
-        <v>25998.8</v>
+        <v>27408.08</v>
       </c>
       <c r="P6" t="n">
-        <v>73938.64</v>
+        <v>74827.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>90735.82000000001</v>
+        <v>95654.21000000001</v>
       </c>
       <c r="R6" t="n">
-        <v>36969.32</v>
+        <v>37313.98</v>
       </c>
       <c r="S6" t="n">
-        <v>42567.13</v>
+        <v>44127.01</v>
       </c>
       <c r="T6" t="n">
-        <v>5597.81</v>
+        <v>6813.03</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1043,37 +1043,37 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1.109936708860759</v>
+        <v>1.3</v>
       </c>
       <c r="K7" t="n">
-        <v>2.219873417721519</v>
+        <v>2.61</v>
       </c>
       <c r="L7" t="n">
-        <v>1.99</v>
+        <v>2.49</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.1036</v>
+        <v>-0.046</v>
       </c>
       <c r="N7" t="n">
         <v>25117</v>
       </c>
       <c r="O7" t="n">
-        <v>35198.45</v>
+        <v>29044.88</v>
       </c>
       <c r="P7" t="n">
-        <v>55756.56063291139</v>
+        <v>65555.37</v>
       </c>
       <c r="Q7" t="n">
-        <v>70044.91</v>
+        <v>72321.75999999999</v>
       </c>
       <c r="R7" t="n">
-        <v>27878.28031645569</v>
+        <v>32903.27</v>
       </c>
       <c r="S7" t="n">
-        <v>30976.86</v>
+        <v>34563.41</v>
       </c>
       <c r="T7" t="n">
-        <v>3098.58</v>
+        <v>1660.14</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -1116,16 +1116,16 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.285625</v>
+        <v>0.28</v>
       </c>
       <c r="K8" t="n">
-        <v>0.57125</v>
+        <v>0.55</v>
       </c>
       <c r="L8" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.0022</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>96560</v>
@@ -1134,16 +1134,16 @@
         <v>96560</v>
       </c>
       <c r="P8" t="n">
-        <v>55159.9</v>
+        <v>53108</v>
       </c>
       <c r="Q8" t="n">
-        <v>55159.9</v>
+        <v>53108</v>
       </c>
       <c r="R8" t="n">
-        <v>27579.95</v>
+        <v>26071.2</v>
       </c>
       <c r="S8" t="n">
-        <v>27579.95</v>
+        <v>26071.2</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
@@ -1189,37 +1189,37 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.6547596153846154</v>
+        <v>0.7</v>
       </c>
       <c r="K9" t="n">
-        <v>1.309519230769231</v>
+        <v>1.4</v>
       </c>
       <c r="L9" t="n">
         <v>1.49</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1378</v>
+        <v>0.0643</v>
       </c>
       <c r="N9" t="n">
         <v>38981</v>
       </c>
       <c r="O9" t="n">
-        <v>29130.58</v>
+        <v>33869.56</v>
       </c>
       <c r="P9" t="n">
-        <v>51046.36913461538</v>
+        <v>54573.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>43404.57</v>
+        <v>50465.65</v>
       </c>
       <c r="R9" t="n">
-        <v>25523.18456730769</v>
+        <v>27286.7</v>
       </c>
       <c r="S9" t="n">
-        <v>24331.04</v>
+        <v>26756.96</v>
       </c>
       <c r="T9" t="n">
-        <v>-1192.14</v>
+        <v>-529.74</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1262,37 +1262,37 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>4.240049019607843</v>
+        <v>4.12</v>
       </c>
       <c r="K10" t="n">
-        <v>8.480098039215687</v>
+        <v>8.24</v>
       </c>
       <c r="L10" t="n">
-        <v>9.49</v>
+        <v>8.99</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1191</v>
+        <v>0.091</v>
       </c>
       <c r="N10" t="n">
         <v>7050</v>
       </c>
       <c r="O10" t="n">
-        <v>5862.85</v>
+        <v>6112.08</v>
       </c>
       <c r="P10" t="n">
-        <v>59784.69117647059</v>
+        <v>58092</v>
       </c>
       <c r="Q10" t="n">
-        <v>55638.42</v>
+        <v>54947.63</v>
       </c>
       <c r="R10" t="n">
-        <v>29892.34558823529</v>
+        <v>29046</v>
       </c>
       <c r="S10" t="n">
-        <v>30779.66</v>
+        <v>29765.84</v>
       </c>
       <c r="T10" t="n">
-        <v>887.3099999999999</v>
+        <v>719.84</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1335,37 +1335,37 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>4.370392156862745</v>
+        <v>4.25</v>
       </c>
       <c r="K11" t="n">
-        <v>8.74078431372549</v>
+        <v>8.5</v>
       </c>
       <c r="L11" t="n">
         <v>7.99</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.0859</v>
+        <v>-0.06</v>
       </c>
       <c r="N11" t="n">
         <v>6945</v>
       </c>
       <c r="O11" t="n">
-        <v>9631.639999999999</v>
+        <v>8700.1</v>
       </c>
       <c r="P11" t="n">
-        <v>60704.74705882352</v>
+        <v>59032.5</v>
       </c>
       <c r="Q11" t="n">
-        <v>76956.77</v>
+        <v>69513.84</v>
       </c>
       <c r="R11" t="n">
-        <v>30352.37352941176</v>
+        <v>29516.25</v>
       </c>
       <c r="S11" t="n">
-        <v>34862.74</v>
+        <v>32538.39</v>
       </c>
       <c r="T11" t="n">
-        <v>4510.37</v>
+        <v>3022.14</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -1408,16 +1408,16 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>5.046902173913042</v>
+        <v>4.97</v>
       </c>
       <c r="K12" t="n">
-        <v>10.09380434782608</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="L12" t="n">
-        <v>10.09</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>7200</v>
@@ -1426,16 +1426,16 @@
         <v>7200</v>
       </c>
       <c r="P12" t="n">
-        <v>72675.39130434781</v>
+        <v>71640</v>
       </c>
       <c r="Q12" t="n">
-        <v>72675.39</v>
+        <v>71640</v>
       </c>
       <c r="R12" t="n">
-        <v>36337.6956521739</v>
+        <v>35856</v>
       </c>
       <c r="S12" t="n">
-        <v>36337.7</v>
+        <v>35856</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1481,37 +1481,37 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.9516504854368931</v>
+        <v>0.82</v>
       </c>
       <c r="K13" t="n">
-        <v>1.903300970873786</v>
+        <v>1.65</v>
       </c>
       <c r="L13" t="n">
-        <v>2.49</v>
+        <v>1.49</v>
       </c>
       <c r="M13" t="n">
-        <v>0.3083</v>
+        <v>-0.097</v>
       </c>
       <c r="N13" t="n">
         <v>29715</v>
       </c>
       <c r="O13" t="n">
-        <v>23261.95</v>
+        <v>32609.17</v>
       </c>
       <c r="P13" t="n">
-        <v>56556.58834951456</v>
+        <v>49029.75</v>
       </c>
       <c r="Q13" t="n">
-        <v>57922.25</v>
+        <v>48587.67</v>
       </c>
       <c r="R13" t="n">
-        <v>28278.29417475728</v>
+        <v>24663.45</v>
       </c>
       <c r="S13" t="n">
-        <v>35785.01</v>
+        <v>21848.15</v>
       </c>
       <c r="T13" t="n">
-        <v>7506.72</v>
+        <v>-2815.3</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -1554,16 +1554,16 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1.486730769230769</v>
+        <v>1.48</v>
       </c>
       <c r="K14" t="n">
-        <v>2.973461538461538</v>
+        <v>2.95</v>
       </c>
       <c r="L14" t="n">
-        <v>2.97</v>
+        <v>2.95</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.0012</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>17999</v>
@@ -1572,16 +1572,16 @@
         <v>17999</v>
       </c>
       <c r="P14" t="n">
-        <v>53519.33423076923</v>
+        <v>53097.05</v>
       </c>
       <c r="Q14" t="n">
-        <v>53519.33</v>
+        <v>53097.05</v>
       </c>
       <c r="R14" t="n">
-        <v>26759.66711538461</v>
+        <v>26458.53</v>
       </c>
       <c r="S14" t="n">
-        <v>26759.67</v>
+        <v>26458.53</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1627,37 +1627,37 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>3.011490384615385</v>
+        <v>3.12</v>
       </c>
       <c r="K15" t="n">
-        <v>6.022980769230769</v>
+        <v>6.25</v>
       </c>
       <c r="L15" t="n">
-        <v>5.49</v>
+        <v>5.99</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.0885</v>
+        <v>-0.0416</v>
       </c>
       <c r="N15" t="n">
         <v>7847</v>
       </c>
       <c r="O15" t="n">
-        <v>13256.87</v>
+        <v>9980.25</v>
       </c>
       <c r="P15" t="n">
-        <v>47262.33009615385</v>
+        <v>49043.75</v>
       </c>
       <c r="Q15" t="n">
-        <v>72780.22</v>
+        <v>59781.69</v>
       </c>
       <c r="R15" t="n">
-        <v>23631.16504807692</v>
+        <v>24561.11</v>
       </c>
       <c r="S15" t="n">
-        <v>32857.28</v>
+        <v>28643.31</v>
       </c>
       <c r="T15" t="n">
-        <v>9226.110000000001</v>
+        <v>4082.2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -1700,37 +1700,37 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>5.561201923076923</v>
+        <v>5.36</v>
       </c>
       <c r="K16" t="n">
-        <v>11.12240384615385</v>
+        <v>10.73</v>
       </c>
       <c r="L16" t="n">
-        <v>10.49</v>
+        <v>9.99</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.0569</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="N16" t="n">
         <v>6290</v>
       </c>
       <c r="O16" t="n">
-        <v>7955.24</v>
+        <v>8378.5</v>
       </c>
       <c r="P16" t="n">
-        <v>69959.92019230769</v>
+        <v>67491.7</v>
       </c>
       <c r="Q16" t="n">
-        <v>83450.50999999999</v>
+        <v>83701.2</v>
       </c>
       <c r="R16" t="n">
-        <v>34979.96009615385</v>
+        <v>33777.3</v>
       </c>
       <c r="S16" t="n">
-        <v>39209.79</v>
+        <v>38792.45</v>
       </c>
       <c r="T16" t="n">
-        <v>4229.83</v>
+        <v>5015.15</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -1773,16 +1773,16 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>1.034558823529412</v>
+        <v>1.04</v>
       </c>
       <c r="K17" t="n">
-        <v>2.069117647058824</v>
+        <v>2.08</v>
       </c>
       <c r="L17" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
         <v>24780</v>
@@ -1791,16 +1791,16 @@
         <v>24780</v>
       </c>
       <c r="P17" t="n">
-        <v>51272.73529411765</v>
+        <v>51542.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>51272.74</v>
+        <v>51542.4</v>
       </c>
       <c r="R17" t="n">
-        <v>25636.36764705883</v>
+        <v>25771.2</v>
       </c>
       <c r="S17" t="n">
-        <v>25636.37</v>
+        <v>25771.2</v>
       </c>
       <c r="T17" t="n">
         <v>0</v>
@@ -1846,37 +1846,37 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>1.083787878787879</v>
+        <v>1.12</v>
       </c>
       <c r="K18" t="n">
-        <v>2.167575757575757</v>
+        <v>2.25</v>
       </c>
       <c r="L18" t="n">
-        <v>1.99</v>
+        <v>2.03</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.0819</v>
+        <v>-0.0978</v>
       </c>
       <c r="N18" t="n">
         <v>25954</v>
       </c>
       <c r="O18" t="n">
-        <v>31680.32</v>
+        <v>32994.04</v>
       </c>
       <c r="P18" t="n">
-        <v>56257.26121212121</v>
+        <v>58396.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>63043.83</v>
+        <v>66977.89999999999</v>
       </c>
       <c r="R18" t="n">
-        <v>28128.6306060606</v>
+        <v>29328.02</v>
       </c>
       <c r="S18" t="n">
-        <v>28709.09</v>
+        <v>30024.58</v>
       </c>
       <c r="T18" t="n">
-        <v>580.46</v>
+        <v>696.5599999999999</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
@@ -1919,37 +1919,37 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>1.085769230769231</v>
+        <v>1.04</v>
       </c>
       <c r="K19" t="n">
-        <v>2.171538461538462</v>
+        <v>2.08</v>
       </c>
       <c r="L19" t="n">
-        <v>2.49</v>
+        <v>1.99</v>
       </c>
       <c r="M19" t="n">
-        <v>0.1467</v>
+        <v>-0.0433</v>
       </c>
       <c r="N19" t="n">
         <v>29503</v>
       </c>
       <c r="O19" t="n">
-        <v>26476.92</v>
+        <v>30553.27</v>
       </c>
       <c r="P19" t="n">
-        <v>64066.89923076923</v>
+        <v>61366.24</v>
       </c>
       <c r="Q19" t="n">
-        <v>65927.53999999999</v>
+        <v>60801</v>
       </c>
       <c r="R19" t="n">
-        <v>32033.44961538462</v>
+        <v>30683.12</v>
       </c>
       <c r="S19" t="n">
-        <v>37179.71</v>
+        <v>29025.6</v>
       </c>
       <c r="T19" t="n">
-        <v>5146.26</v>
+        <v>-1657.52</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -1992,37 +1992,37 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>1.784047619047619</v>
+        <v>1.48</v>
       </c>
       <c r="K20" t="n">
-        <v>3.568095238095238</v>
+        <v>2.95</v>
       </c>
       <c r="L20" t="n">
-        <v>3.49</v>
+        <v>2.99</v>
       </c>
       <c r="M20" t="n">
-        <v>-0.0219</v>
+        <v>0.0136</v>
       </c>
       <c r="N20" t="n">
         <v>36581</v>
       </c>
       <c r="O20" t="n">
-        <v>38341.18</v>
+        <v>35549.56</v>
       </c>
       <c r="P20" t="n">
-        <v>130524.4919047619</v>
+        <v>107913.95</v>
       </c>
       <c r="Q20" t="n">
-        <v>133810.73</v>
+        <v>106293.19</v>
       </c>
       <c r="R20" t="n">
-        <v>65262.24595238095</v>
+        <v>53774.07</v>
       </c>
       <c r="S20" t="n">
-        <v>65408.23</v>
+        <v>53679.84</v>
       </c>
       <c r="T20" t="n">
-        <v>145.98</v>
+        <v>-94.23</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -2065,37 +2065,37 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1.551586538461539</v>
+        <v>1.6</v>
       </c>
       <c r="K21" t="n">
-        <v>3.103173076923077</v>
+        <v>3.19</v>
       </c>
       <c r="L21" t="n">
         <v>3.49</v>
       </c>
       <c r="M21" t="n">
-        <v>0.1247</v>
+        <v>0.094</v>
       </c>
       <c r="N21" t="n">
         <v>16808</v>
       </c>
       <c r="O21" t="n">
-        <v>14754.87</v>
+        <v>15213.41</v>
       </c>
       <c r="P21" t="n">
-        <v>52158.13307692308</v>
+        <v>53617.52</v>
       </c>
       <c r="Q21" t="n">
-        <v>51494.51</v>
+        <v>53094.79</v>
       </c>
       <c r="R21" t="n">
-        <v>26079.06653846154</v>
+        <v>26724.72</v>
       </c>
       <c r="S21" t="n">
-        <v>28601.05</v>
+        <v>28753.34</v>
       </c>
       <c r="T21" t="n">
-        <v>2521.98</v>
+        <v>2028.62</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -2138,37 +2138,37 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>2.692029702970297</v>
+        <v>2.48</v>
       </c>
       <c r="K22" t="n">
-        <v>5.384059405940594</v>
+        <v>4.95</v>
       </c>
       <c r="L22" t="n">
-        <v>5.49</v>
+        <v>4.99</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0197</v>
+        <v>0.0081</v>
       </c>
       <c r="N22" t="n">
         <v>10218</v>
       </c>
       <c r="O22" t="n">
-        <v>9844.639999999999</v>
+        <v>10062.1</v>
       </c>
       <c r="P22" t="n">
-        <v>55014.31900990099</v>
+        <v>50579.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>54047.09</v>
+        <v>50209.89</v>
       </c>
       <c r="R22" t="n">
-        <v>27507.15950495049</v>
+        <v>25238.46</v>
       </c>
       <c r="S22" t="n">
-        <v>27545.02</v>
+        <v>25255.88</v>
       </c>
       <c r="T22" t="n">
-        <v>37.86</v>
+        <v>17.42</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -2211,37 +2211,37 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>2.740288461538462</v>
+        <v>2.48</v>
       </c>
       <c r="K23" t="n">
-        <v>5.480576923076923</v>
+        <v>4.95</v>
       </c>
       <c r="L23" t="n">
-        <v>6.49</v>
+        <v>4.99</v>
       </c>
       <c r="M23" t="n">
-        <v>0.1842</v>
+        <v>0.0081</v>
       </c>
       <c r="N23" t="n">
         <v>11556</v>
       </c>
       <c r="O23" t="n">
-        <v>9679.610000000001</v>
+        <v>11458.93</v>
       </c>
       <c r="P23" t="n">
-        <v>63333.54692307693</v>
+        <v>57202.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>62820.64</v>
+        <v>57180.06</v>
       </c>
       <c r="R23" t="n">
-        <v>31666.77346153847</v>
+        <v>28543.32</v>
       </c>
       <c r="S23" t="n">
-        <v>36295.73</v>
+        <v>28761.91</v>
       </c>
       <c r="T23" t="n">
-        <v>4628.96</v>
+        <v>218.59</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
@@ -2284,37 +2284,37 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>2.273269230769231</v>
+        <v>2.12</v>
       </c>
       <c r="K24" t="n">
-        <v>4.546538461538462</v>
+        <v>4.25</v>
       </c>
       <c r="L24" t="n">
-        <v>4.49</v>
+        <v>3.99</v>
       </c>
       <c r="M24" t="n">
-        <v>-0.0124</v>
+        <v>-0.0612</v>
       </c>
       <c r="N24" t="n">
         <v>12462</v>
       </c>
       <c r="O24" t="n">
-        <v>12834.02</v>
+        <v>14455.55</v>
       </c>
       <c r="P24" t="n">
-        <v>56658.96230769231</v>
+        <v>52963.5</v>
       </c>
       <c r="Q24" t="n">
-        <v>57624.75</v>
+        <v>57677.64</v>
       </c>
       <c r="R24" t="n">
-        <v>28329.48115384615</v>
+        <v>26544.06</v>
       </c>
       <c r="S24" t="n">
-        <v>28449.57</v>
+        <v>27031.88</v>
       </c>
       <c r="T24" t="n">
-        <v>120.09</v>
+        <v>487.82</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -2357,37 +2357,37 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>2.580148514851485</v>
+        <v>2.48</v>
       </c>
       <c r="K25" t="n">
-        <v>5.160297029702971</v>
+        <v>4.95</v>
       </c>
       <c r="L25" t="n">
         <v>4.49</v>
       </c>
       <c r="M25" t="n">
-        <v>-0.1299</v>
+        <v>-0.0929</v>
       </c>
       <c r="N25" t="n">
         <v>10675</v>
       </c>
       <c r="O25" t="n">
-        <v>16753.57</v>
+        <v>14641.2</v>
       </c>
       <c r="P25" t="n">
-        <v>55086.17079207921</v>
+        <v>52841.25</v>
       </c>
       <c r="Q25" t="n">
-        <v>75223.53999999999</v>
+        <v>65738.99000000001</v>
       </c>
       <c r="R25" t="n">
-        <v>27543.08539603961</v>
+        <v>26367.25</v>
       </c>
       <c r="S25" t="n">
-        <v>31996.84</v>
+        <v>29428.81</v>
       </c>
       <c r="T25" t="n">
-        <v>4453.75</v>
+        <v>3061.56</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -2430,37 +2430,37 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0.6933653846153847</v>
+        <v>0.98</v>
       </c>
       <c r="K26" t="n">
-        <v>1.386730769230769</v>
+        <v>1.95</v>
       </c>
       <c r="L26" t="n">
-        <v>1.49</v>
+        <v>1.99</v>
       </c>
       <c r="M26" t="n">
-        <v>0.0745</v>
+        <v>0.0205</v>
       </c>
       <c r="N26" t="n">
         <v>40748</v>
       </c>
       <c r="O26" t="n">
-        <v>37343.21</v>
+        <v>39755.17</v>
       </c>
       <c r="P26" t="n">
-        <v>56506.50538461539</v>
+        <v>79458.60000000001</v>
       </c>
       <c r="Q26" t="n">
-        <v>55641.39</v>
+        <v>79112.78999999999</v>
       </c>
       <c r="R26" t="n">
-        <v>28253.25269230769</v>
+        <v>39525.56</v>
       </c>
       <c r="S26" t="n">
-        <v>29748.9</v>
+        <v>40152.72</v>
       </c>
       <c r="T26" t="n">
-        <v>1495.65</v>
+        <v>627.16</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>0.4440865384615385</v>
+        <v>0.42</v>
       </c>
       <c r="K27" t="n">
-        <v>0.888173076923077</v>
+        <v>0.85</v>
       </c>
       <c r="L27" t="n">
-        <v>0.89</v>
+        <v>0.85</v>
       </c>
       <c r="M27" t="n">
-        <v>0.0021</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
         <v>89898</v>
@@ -2521,19 +2521,19 @@
         <v>89898</v>
       </c>
       <c r="P27" t="n">
-        <v>79844.98326923078</v>
+        <v>76413.3</v>
       </c>
       <c r="Q27" t="n">
-        <v>79844.98</v>
+        <v>76413.3</v>
       </c>
       <c r="R27" t="n">
-        <v>39922.49163461539</v>
+        <v>38656.14</v>
       </c>
       <c r="S27" t="n">
-        <v>39922.49</v>
+        <v>38656.14</v>
       </c>
       <c r="T27" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
@@ -2576,16 +2576,16 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>1.490578947368421</v>
+        <v>1.48</v>
       </c>
       <c r="K28" t="n">
-        <v>2.981157894736842</v>
+        <v>2.95</v>
       </c>
       <c r="L28" t="n">
-        <v>2.98</v>
+        <v>2.95</v>
       </c>
       <c r="M28" t="n">
-        <v>-0.0004</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
         <v>15690</v>
@@ -2594,19 +2594,19 @@
         <v>15690</v>
       </c>
       <c r="P28" t="n">
-        <v>46774.36736842106</v>
+        <v>46285.5</v>
       </c>
       <c r="Q28" t="n">
-        <v>46774.37</v>
+        <v>46285.5</v>
       </c>
       <c r="R28" t="n">
-        <v>23387.18368421053</v>
+        <v>23064.3</v>
       </c>
       <c r="S28" t="n">
-        <v>23387.18</v>
+        <v>23064.3</v>
       </c>
       <c r="T28" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -2649,16 +2649,16 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0.4594230769230769</v>
+        <v>0.46</v>
       </c>
       <c r="K29" t="n">
-        <v>0.9188461538461539</v>
+        <v>0.92</v>
       </c>
       <c r="L29" t="n">
         <v>0.92</v>
       </c>
       <c r="M29" t="n">
-        <v>0.0013</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>32692</v>
@@ -2667,16 +2667,16 @@
         <v>32692</v>
       </c>
       <c r="P29" t="n">
-        <v>30038.91846153846</v>
+        <v>30076.64</v>
       </c>
       <c r="Q29" t="n">
-        <v>30038.92</v>
+        <v>30076.64</v>
       </c>
       <c r="R29" t="n">
-        <v>15019.45923076923</v>
+        <v>15038.32</v>
       </c>
       <c r="S29" t="n">
-        <v>15019.46</v>
+        <v>15038.32</v>
       </c>
       <c r="T29" t="n">
         <v>0</v>
@@ -2722,37 +2722,37 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>1.042886597938144</v>
+        <v>1.04</v>
       </c>
       <c r="K30" t="n">
-        <v>2.085773195876289</v>
+        <v>2.08</v>
       </c>
       <c r="L30" t="n">
-        <v>2.49</v>
+        <v>1.99</v>
       </c>
       <c r="M30" t="n">
-        <v>0.1938</v>
+        <v>-0.0433</v>
       </c>
       <c r="N30" t="n">
         <v>39840</v>
       </c>
       <c r="O30" t="n">
-        <v>30353.25</v>
+        <v>42639.57</v>
       </c>
       <c r="P30" t="n">
-        <v>83097.20412371134</v>
+        <v>82867.2</v>
       </c>
       <c r="Q30" t="n">
-        <v>75579.60000000001</v>
+        <v>84852.75</v>
       </c>
       <c r="R30" t="n">
-        <v>41548.60206185567</v>
+        <v>41433.6</v>
       </c>
       <c r="S30" t="n">
-        <v>43924.6</v>
+        <v>40507.59</v>
       </c>
       <c r="T30" t="n">
-        <v>2376</v>
+        <v>-926.01</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -2795,16 +2795,16 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>1.046134020618557</v>
+        <v>1.04</v>
       </c>
       <c r="K31" t="n">
-        <v>2.092268041237113</v>
+        <v>2.08</v>
       </c>
       <c r="L31" t="n">
-        <v>2.09</v>
+        <v>2.08</v>
       </c>
       <c r="M31" t="n">
-        <v>-0.0011</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>27732</v>
@@ -2813,16 +2813,16 @@
         <v>27732</v>
       </c>
       <c r="P31" t="n">
-        <v>58022.77731958762</v>
+        <v>57682.56</v>
       </c>
       <c r="Q31" t="n">
-        <v>58022.78</v>
+        <v>57682.56</v>
       </c>
       <c r="R31" t="n">
-        <v>29011.38865979381</v>
+        <v>28841.28</v>
       </c>
       <c r="S31" t="n">
-        <v>29011.39</v>
+        <v>28841.28</v>
       </c>
       <c r="T31" t="n">
         <v>0</v>
@@ -2868,37 +2868,37 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>6.445777777777778</v>
+        <v>6.38</v>
       </c>
       <c r="K32" t="n">
-        <v>12.89155555555556</v>
+        <v>12.75</v>
       </c>
       <c r="L32" t="n">
         <v>11.49</v>
       </c>
       <c r="M32" t="n">
-        <v>-0.1087</v>
+        <v>-0.0988</v>
       </c>
       <c r="N32" t="n">
         <v>27577</v>
       </c>
       <c r="O32" t="n">
-        <v>41079.12</v>
+        <v>39538.29</v>
       </c>
       <c r="P32" t="n">
-        <v>355510.4275555555</v>
+        <v>351606.75</v>
       </c>
       <c r="Q32" t="n">
-        <v>471999.06</v>
+        <v>454295.01</v>
       </c>
       <c r="R32" t="n">
-        <v>177755.2137777778</v>
+        <v>175665.49</v>
       </c>
       <c r="S32" t="n">
-        <v>207212.2</v>
+        <v>202040.69</v>
       </c>
       <c r="T32" t="n">
-        <v>29456.99</v>
+        <v>26375.2</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
@@ -2941,37 +2941,37 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>1.526627906976744</v>
+        <v>1.48</v>
       </c>
       <c r="K33" t="n">
-        <v>3.053255813953489</v>
+        <v>2.95</v>
       </c>
       <c r="L33" t="n">
         <v>2.99</v>
       </c>
       <c r="M33" t="n">
-        <v>-0.0207</v>
+        <v>0.0136</v>
       </c>
       <c r="N33" t="n">
         <v>15771</v>
       </c>
       <c r="O33" t="n">
-        <v>16987.75</v>
+        <v>15034.7</v>
       </c>
       <c r="P33" t="n">
-        <v>48152.89744186047</v>
+        <v>46524.45</v>
       </c>
       <c r="Q33" t="n">
-        <v>50793.37</v>
+        <v>44953.74</v>
       </c>
       <c r="R33" t="n">
-        <v>24076.44872093024</v>
+        <v>23183.37</v>
       </c>
       <c r="S33" t="n">
-        <v>24859.4</v>
+        <v>22702.39</v>
       </c>
       <c r="T33" t="n">
-        <v>782.95</v>
+        <v>-480.98</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
@@ -3014,37 +3014,37 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.8851923076923077</v>
+        <v>0.82</v>
       </c>
       <c r="K34" t="n">
-        <v>1.770384615384615</v>
+        <v>1.65</v>
       </c>
       <c r="L34" t="n">
         <v>1.49</v>
       </c>
       <c r="M34" t="n">
-        <v>-0.1584</v>
+        <v>-0.097</v>
       </c>
       <c r="N34" t="n">
         <v>29037</v>
       </c>
       <c r="O34" t="n">
-        <v>51383.54</v>
+        <v>40699.2</v>
       </c>
       <c r="P34" t="n">
-        <v>51406.65807692308</v>
+        <v>47911.05</v>
       </c>
       <c r="Q34" t="n">
-        <v>76561.47</v>
+        <v>60641.81</v>
       </c>
       <c r="R34" t="n">
-        <v>25703.32903846154</v>
+        <v>24100.71</v>
       </c>
       <c r="S34" t="n">
-        <v>31077.16</v>
+        <v>27268.47</v>
       </c>
       <c r="T34" t="n">
-        <v>5373.83</v>
+        <v>3167.76</v>
       </c>
       <c r="U34" t="inlineStr">
         <is>
@@ -3087,37 +3087,37 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>1.513441558441559</v>
+        <v>1.48</v>
       </c>
       <c r="K35" t="n">
-        <v>3.026883116883117</v>
+        <v>2.95</v>
       </c>
       <c r="L35" t="n">
         <v>2.99</v>
       </c>
       <c r="M35" t="n">
-        <v>-0.0122</v>
+        <v>0.0136</v>
       </c>
       <c r="N35" t="n">
         <v>18551</v>
       </c>
       <c r="O35" t="n">
-        <v>19024.29</v>
+        <v>18044.63</v>
       </c>
       <c r="P35" t="n">
-        <v>56151.7087012987</v>
+        <v>54725.45</v>
       </c>
       <c r="Q35" t="n">
-        <v>56882.64</v>
+        <v>53953.43</v>
       </c>
       <c r="R35" t="n">
-        <v>28075.85435064935</v>
+        <v>27269.97</v>
       </c>
       <c r="S35" t="n">
-        <v>28090.48</v>
+        <v>27247.38</v>
       </c>
       <c r="T35" t="n">
-        <v>14.63</v>
+        <v>-22.59</v>
       </c>
       <c r="U35" t="inlineStr">
         <is>
@@ -3160,37 +3160,37 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>3.273478260869565</v>
+        <v>3.82</v>
       </c>
       <c r="K36" t="n">
-        <v>6.546956521739131</v>
+        <v>7.64</v>
       </c>
       <c r="L36" t="n">
-        <v>7.49</v>
+        <v>7.99</v>
       </c>
       <c r="M36" t="n">
-        <v>0.144</v>
+        <v>0.0458</v>
       </c>
       <c r="N36" t="n">
         <v>3869</v>
       </c>
       <c r="O36" t="n">
-        <v>3251.03</v>
+        <v>3651.25</v>
       </c>
       <c r="P36" t="n">
-        <v>25330.1747826087</v>
+        <v>29559.16</v>
       </c>
       <c r="Q36" t="n">
-        <v>24350.22</v>
+        <v>29173.49</v>
       </c>
       <c r="R36" t="n">
-        <v>12665.08739130435</v>
+        <v>14779.58</v>
       </c>
       <c r="S36" t="n">
-        <v>13708.04</v>
+        <v>15225.71</v>
       </c>
       <c r="T36" t="n">
-        <v>1042.95</v>
+        <v>446.13</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
@@ -3233,37 +3233,37 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>1.7274</v>
+        <v>1.48</v>
       </c>
       <c r="K37" t="n">
-        <v>3.4548</v>
+        <v>2.95</v>
       </c>
       <c r="L37" t="n">
-        <v>3.49</v>
+        <v>2.99</v>
       </c>
       <c r="M37" t="n">
-        <v>0.0102</v>
+        <v>0.0136</v>
       </c>
       <c r="N37" t="n">
         <v>19597</v>
       </c>
       <c r="O37" t="n">
-        <v>18987.39</v>
+        <v>18791.24</v>
       </c>
       <c r="P37" t="n">
-        <v>67703.7156</v>
+        <v>57811.15</v>
       </c>
       <c r="Q37" t="n">
-        <v>66265.98</v>
+        <v>56185.8</v>
       </c>
       <c r="R37" t="n">
-        <v>33851.8578</v>
+        <v>28807.59</v>
       </c>
       <c r="S37" t="n">
-        <v>33467.17</v>
+        <v>28374.77</v>
       </c>
       <c r="T37" t="n">
-        <v>-384.69</v>
+        <v>-432.82</v>
       </c>
       <c r="U37" t="inlineStr">
         <is>
@@ -3306,37 +3306,37 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>2.635145631067962</v>
+        <v>2.48</v>
       </c>
       <c r="K38" t="n">
-        <v>5.270291262135923</v>
+        <v>4.95</v>
       </c>
       <c r="L38" t="n">
-        <v>5.49</v>
+        <v>4.49</v>
       </c>
       <c r="M38" t="n">
-        <v>0.0417</v>
+        <v>-0.0929</v>
       </c>
       <c r="N38" t="n">
         <v>28378</v>
       </c>
       <c r="O38" t="n">
-        <v>26047.83</v>
+        <v>34821.08</v>
       </c>
       <c r="P38" t="n">
-        <v>149560.3254368932</v>
+        <v>140471.1</v>
       </c>
       <c r="Q38" t="n">
-        <v>143002.6</v>
+        <v>156346.63</v>
       </c>
       <c r="R38" t="n">
-        <v>74780.16271844661</v>
+        <v>70093.66</v>
       </c>
       <c r="S38" t="n">
-        <v>74362.77</v>
+        <v>69990.36</v>
       </c>
       <c r="T38" t="n">
-        <v>-417.39</v>
+        <v>-103.3</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
@@ -3379,37 +3379,37 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>3.906274509803922</v>
+        <v>4.12</v>
       </c>
       <c r="K39" t="n">
-        <v>7.812549019607843</v>
+        <v>8.25</v>
       </c>
       <c r="L39" t="n">
         <v>7.49</v>
       </c>
       <c r="M39" t="n">
-        <v>-0.0413</v>
+        <v>-0.0921</v>
       </c>
       <c r="N39" t="n">
         <v>10175</v>
       </c>
       <c r="O39" t="n">
-        <v>12911.6</v>
+        <v>17565.15</v>
       </c>
       <c r="P39" t="n">
-        <v>79492.6862745098</v>
+        <v>83943.75</v>
       </c>
       <c r="Q39" t="n">
-        <v>96707.92</v>
+        <v>131562.95</v>
       </c>
       <c r="R39" t="n">
-        <v>39746.3431372549</v>
+        <v>42022.75</v>
       </c>
       <c r="S39" t="n">
-        <v>46271.65</v>
+        <v>59194.54</v>
       </c>
       <c r="T39" t="n">
-        <v>6525.31</v>
+        <v>17171.79</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
@@ -3452,37 +3452,37 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>4.220817307692308</v>
+        <v>4.49</v>
       </c>
       <c r="K40" t="n">
-        <v>8.441634615384617</v>
+        <v>8.98</v>
       </c>
       <c r="L40" t="n">
-        <v>8.49</v>
+        <v>9.49</v>
       </c>
       <c r="M40" t="n">
-        <v>0.0057</v>
+        <v>0.0568</v>
       </c>
       <c r="N40" t="n">
         <v>6862</v>
       </c>
       <c r="O40" t="n">
-        <v>6786.35</v>
+        <v>6164.54</v>
       </c>
       <c r="P40" t="n">
-        <v>57926.49673076924</v>
+        <v>61620.76</v>
       </c>
       <c r="Q40" t="n">
-        <v>57616.12</v>
+        <v>58501.5</v>
       </c>
       <c r="R40" t="n">
-        <v>28963.24836538462</v>
+        <v>30810.38</v>
       </c>
       <c r="S40" t="n">
-        <v>28972.17</v>
+        <v>30822.71</v>
       </c>
       <c r="T40" t="n">
-        <v>8.92</v>
+        <v>12.33</v>
       </c>
       <c r="U40" t="inlineStr">
         <is>
@@ -3525,37 +3525,37 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>3.969742268041237</v>
+        <v>4.12</v>
       </c>
       <c r="K41" t="n">
-        <v>7.939484536082475</v>
+        <v>8.25</v>
       </c>
       <c r="L41" t="n">
         <v>7.49</v>
       </c>
       <c r="M41" t="n">
-        <v>-0.0566</v>
+        <v>-0.0921</v>
       </c>
       <c r="N41" t="n">
         <v>7425</v>
       </c>
       <c r="O41" t="n">
-        <v>9994.59</v>
+        <v>12154.28</v>
       </c>
       <c r="P41" t="n">
-        <v>58950.67268041238</v>
+        <v>61256.25</v>
       </c>
       <c r="Q41" t="n">
-        <v>74859.44</v>
+        <v>91035.53999999999</v>
       </c>
       <c r="R41" t="n">
-        <v>29475.33634020619</v>
+        <v>30665.25</v>
       </c>
       <c r="S41" t="n">
-        <v>35183.52</v>
+        <v>40959.91</v>
       </c>
       <c r="T41" t="n">
-        <v>5708.18</v>
+        <v>10294.66</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
@@ -3598,37 +3598,37 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>3.936346153846154</v>
+        <v>4.37</v>
       </c>
       <c r="K42" t="n">
-        <v>7.872692307692308</v>
+        <v>8.74</v>
       </c>
       <c r="L42" t="n">
-        <v>7.49</v>
+        <v>7.99</v>
       </c>
       <c r="M42" t="n">
-        <v>-0.0486</v>
+        <v>-0.0858</v>
       </c>
       <c r="N42" t="n">
         <v>7847</v>
       </c>
       <c r="O42" t="n">
-        <v>9505.469999999999</v>
+        <v>11082.25</v>
       </c>
       <c r="P42" t="n">
-        <v>61777.01653846154</v>
+        <v>68582.78</v>
       </c>
       <c r="Q42" t="n">
-        <v>71195.95</v>
+        <v>88547.17999999999</v>
       </c>
       <c r="R42" t="n">
-        <v>30888.50826923077</v>
+        <v>34291.39</v>
       </c>
       <c r="S42" t="n">
-        <v>33779.14</v>
+        <v>40117.75</v>
       </c>
       <c r="T42" t="n">
-        <v>2890.63</v>
+        <v>5826.36</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
@@ -3671,37 +3671,37 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1.733011363636364</v>
+        <v>1.98</v>
       </c>
       <c r="K43" t="n">
-        <v>3.466022727272727</v>
+        <v>3.95</v>
       </c>
       <c r="L43" t="n">
-        <v>3.49</v>
+        <v>3.99</v>
       </c>
       <c r="M43" t="n">
-        <v>0.0069</v>
+        <v>0.0101</v>
       </c>
       <c r="N43" t="n">
         <v>15727</v>
       </c>
       <c r="O43" t="n">
-        <v>15341.55</v>
+        <v>15166.86</v>
       </c>
       <c r="P43" t="n">
-        <v>54510.13943181818</v>
+        <v>62121.65</v>
       </c>
       <c r="Q43" t="n">
-        <v>53542.01</v>
+        <v>60515.77</v>
       </c>
       <c r="R43" t="n">
-        <v>27255.06971590909</v>
+        <v>30982.19</v>
       </c>
       <c r="S43" t="n">
-        <v>26954.93</v>
+        <v>30485.39</v>
       </c>
       <c r="T43" t="n">
-        <v>-300.14</v>
+        <v>-496.8</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
@@ -3744,37 +3744,37 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>2.802422680412371</v>
+        <v>2.88</v>
       </c>
       <c r="K44" t="n">
-        <v>5.604845360824742</v>
+        <v>5.75</v>
       </c>
       <c r="L44" t="n">
         <v>5.49</v>
       </c>
       <c r="M44" t="n">
-        <v>-0.0205</v>
+        <v>-0.0452</v>
       </c>
       <c r="N44" t="n">
         <v>16840</v>
       </c>
       <c r="O44" t="n">
-        <v>17609.65</v>
+        <v>18608.88</v>
       </c>
       <c r="P44" t="n">
-        <v>94385.59587628864</v>
+        <v>96830</v>
       </c>
       <c r="Q44" t="n">
-        <v>96676.97</v>
+        <v>102162.75</v>
       </c>
       <c r="R44" t="n">
-        <v>47192.79793814432</v>
+        <v>48330.8</v>
       </c>
       <c r="S44" t="n">
-        <v>47327.29</v>
+        <v>48569.18</v>
       </c>
       <c r="T44" t="n">
-        <v>134.49</v>
+        <v>238.38</v>
       </c>
       <c r="U44" t="inlineStr">
         <is>
@@ -3817,16 +3817,16 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>3.602873563218391</v>
+        <v>3.98</v>
       </c>
       <c r="K45" t="n">
-        <v>7.205747126436782</v>
+        <v>7.95</v>
       </c>
       <c r="L45" t="n">
-        <v>7.21</v>
+        <v>7.95</v>
       </c>
       <c r="M45" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
         <v>11054</v>
@@ -3835,19 +3835,19 @@
         <v>11054</v>
       </c>
       <c r="P45" t="n">
-        <v>79652.32873563218</v>
+        <v>87879.3</v>
       </c>
       <c r="Q45" t="n">
-        <v>79652.33</v>
+        <v>87879.3</v>
       </c>
       <c r="R45" t="n">
-        <v>39826.16436781609</v>
+        <v>43884.38</v>
       </c>
       <c r="S45" t="n">
-        <v>39826.16</v>
+        <v>43884.38</v>
       </c>
       <c r="T45" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U45" t="inlineStr">
         <is>
@@ -3890,37 +3890,37 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>2.459020618556701</v>
+        <v>2.12</v>
       </c>
       <c r="K46" t="n">
-        <v>4.918041237113402</v>
+        <v>4.25</v>
       </c>
       <c r="L46" t="n">
-        <v>4.49</v>
+        <v>3.99</v>
       </c>
       <c r="M46" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.0612</v>
       </c>
       <c r="N46" t="n">
         <v>11830</v>
       </c>
       <c r="O46" t="n">
-        <v>15185.71</v>
+        <v>14066</v>
       </c>
       <c r="P46" t="n">
-        <v>58180.42783505155</v>
+        <v>50277.5</v>
       </c>
       <c r="Q46" t="n">
-        <v>68183.86</v>
+        <v>56123.32</v>
       </c>
       <c r="R46" t="n">
-        <v>29090.21391752578</v>
+        <v>25197.9</v>
       </c>
       <c r="S46" t="n">
-        <v>30841.87</v>
+        <v>26303.41</v>
       </c>
       <c r="T46" t="n">
-        <v>1751.66</v>
+        <v>1105.51</v>
       </c>
       <c r="U46" t="inlineStr">
         <is>
@@ -3963,37 +3963,37 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>1.739155844155844</v>
+        <v>1.27</v>
       </c>
       <c r="K47" t="n">
-        <v>3.478311688311688</v>
+        <v>2.55</v>
       </c>
       <c r="L47" t="n">
-        <v>3.99</v>
+        <v>2.49</v>
       </c>
       <c r="M47" t="n">
-        <v>0.1471</v>
+        <v>-0.0235</v>
       </c>
       <c r="N47" t="n">
         <v>32525</v>
       </c>
       <c r="O47" t="n">
-        <v>26055.33</v>
+        <v>33800.89</v>
       </c>
       <c r="P47" t="n">
-        <v>113132.0876623377</v>
+        <v>82938.75</v>
       </c>
       <c r="Q47" t="n">
-        <v>103960.77</v>
+        <v>84164.21000000001</v>
       </c>
       <c r="R47" t="n">
-        <v>56566.04383116883</v>
+        <v>41632</v>
       </c>
       <c r="S47" t="n">
-        <v>58646.49</v>
+        <v>41237.08</v>
       </c>
       <c r="T47" t="n">
-        <v>2080.45</v>
+        <v>-394.92</v>
       </c>
       <c r="U47" t="inlineStr">
         <is>
@@ -4036,37 +4036,37 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>0.6775961538461538</v>
+        <v>0.62</v>
       </c>
       <c r="K48" t="n">
-        <v>1.355192307692308</v>
+        <v>1.25</v>
       </c>
       <c r="L48" t="n">
-        <v>1.49</v>
+        <v>1.37</v>
       </c>
       <c r="M48" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="N48" t="n">
         <v>38064</v>
       </c>
       <c r="O48" t="n">
-        <v>33579.93</v>
+        <v>33720.72</v>
       </c>
       <c r="P48" t="n">
-        <v>51584.03999999999</v>
+        <v>47580</v>
       </c>
       <c r="Q48" t="n">
-        <v>50034.09</v>
+        <v>46197.38</v>
       </c>
       <c r="R48" t="n">
-        <v>25792.02</v>
+        <v>23980.32</v>
       </c>
       <c r="S48" t="n">
-        <v>27280.46</v>
+        <v>25290.54</v>
       </c>
       <c r="T48" t="n">
-        <v>1488.44</v>
+        <v>1310.22</v>
       </c>
       <c r="U48" t="inlineStr">
         <is>
@@ -4109,16 +4109,16 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>1.008365384615385</v>
+        <v>1.04</v>
       </c>
       <c r="K49" t="n">
-        <v>2.016730769230769</v>
+        <v>2.08</v>
       </c>
       <c r="L49" t="n">
-        <v>2.02</v>
+        <v>2.08</v>
       </c>
       <c r="M49" t="n">
-        <v>0.0016</v>
+        <v>0</v>
       </c>
       <c r="N49" t="n">
         <v>98349</v>
@@ -4127,16 +4127,16 @@
         <v>98349</v>
       </c>
       <c r="P49" t="n">
-        <v>198343.4544230769</v>
+        <v>204565.92</v>
       </c>
       <c r="Q49" t="n">
-        <v>198343.45</v>
+        <v>204565.92</v>
       </c>
       <c r="R49" t="n">
-        <v>99171.72721153845</v>
+        <v>102282.96</v>
       </c>
       <c r="S49" t="n">
-        <v>99171.73</v>
+        <v>102282.96</v>
       </c>
       <c r="T49" t="n">
         <v>0</v>
@@ -4182,16 +4182,16 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>1.062307692307692</v>
+        <v>1.08</v>
       </c>
       <c r="K50" t="n">
-        <v>2.124615384615385</v>
+        <v>2.16</v>
       </c>
       <c r="L50" t="n">
-        <v>2.12</v>
+        <v>2.16</v>
       </c>
       <c r="M50" t="n">
-        <v>-0.0022</v>
+        <v>0</v>
       </c>
       <c r="N50" t="n">
         <v>31249</v>
@@ -4200,19 +4200,19 @@
         <v>31249</v>
       </c>
       <c r="P50" t="n">
-        <v>66392.10615384617</v>
+        <v>67497.84</v>
       </c>
       <c r="Q50" t="n">
-        <v>66392.11</v>
+        <v>67497.84</v>
       </c>
       <c r="R50" t="n">
-        <v>33196.05307692308</v>
+        <v>33748.92</v>
       </c>
       <c r="S50" t="n">
-        <v>33196.05</v>
+        <v>33748.92</v>
       </c>
       <c r="T50" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="U50" t="inlineStr">
         <is>
@@ -4255,37 +4255,37 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>1.016359223300971</v>
+        <v>1.04</v>
       </c>
       <c r="K51" t="n">
-        <v>2.032718446601942</v>
+        <v>2.08</v>
       </c>
       <c r="L51" t="n">
         <v>1.99</v>
       </c>
       <c r="M51" t="n">
-        <v>-0.021</v>
+        <v>-0.0433</v>
       </c>
       <c r="N51" t="n">
         <v>37124</v>
       </c>
       <c r="O51" t="n">
-        <v>39197.59</v>
+        <v>41573.23</v>
       </c>
       <c r="P51" t="n">
-        <v>75462.63961165048</v>
+        <v>77217.92</v>
       </c>
       <c r="Q51" t="n">
-        <v>78003.2</v>
+        <v>82730.74000000001</v>
       </c>
       <c r="R51" t="n">
-        <v>37731.31980582524</v>
+        <v>38608.96</v>
       </c>
       <c r="S51" t="n">
-        <v>38164.37</v>
+        <v>39494.57</v>
       </c>
       <c r="T51" t="n">
-        <v>433.05</v>
+        <v>885.61</v>
       </c>
       <c r="U51" t="inlineStr">
         <is>
@@ -4349,16 +4349,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2195980.26</v>
+        <v>2174918.07</v>
       </c>
       <c r="D2" t="n">
-        <v>2363397.08</v>
+        <v>2335043.93</v>
       </c>
       <c r="E2" t="n">
-        <v>167416.84</v>
+        <v>160125.86</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0762</v>
+        <v>0.0736</v>
       </c>
     </row>
     <row r="3">
@@ -4371,16 +4371,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1829983.55</v>
+        <v>1811967.34</v>
       </c>
       <c r="D3" t="n">
-        <v>1952996.32</v>
+        <v>1914692.33</v>
       </c>
       <c r="E3" t="n">
-        <v>123012.77</v>
+        <v>102724.99</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0672</v>
+        <v>0.0567</v>
       </c>
     </row>
     <row r="4">
@@ -4393,16 +4393,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1463986.84</v>
+        <v>1449089.94</v>
       </c>
       <c r="D4" t="n">
-        <v>1556026.62</v>
+        <v>1501367.65</v>
       </c>
       <c r="E4" t="n">
-        <v>92039.77</v>
+        <v>52277.71</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0629</v>
+        <v>0.0361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(pricing): update PROGRESS.md with directional rounding & LLM rejection analysis
</commit_message>
<xml_diff>
--- a/outputs/pricing/pricing_optimization.xlsx
+++ b/outputs/pricing/pricing_optimization.xlsx
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1914692.33</v>
+        <v>1946464.1</v>
       </c>
     </row>
     <row r="6">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>102724.99</v>
+        <v>134496.76</v>
       </c>
     </row>
     <row r="7">
@@ -488,7 +488,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5.67 %</t>
+          <t>7.42 %</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -830,31 +830,31 @@
         <v>1.65</v>
       </c>
       <c r="L4" t="n">
-        <v>1.49</v>
+        <v>1.81</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.097</v>
+        <v>0.097</v>
       </c>
       <c r="N4" t="n">
         <v>40942</v>
       </c>
       <c r="O4" t="n">
-        <v>49332.87</v>
+        <v>34570.15</v>
       </c>
       <c r="P4" t="n">
         <v>67554.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>73505.97</v>
+        <v>62571.98</v>
       </c>
       <c r="R4" t="n">
         <v>33981.86</v>
       </c>
       <c r="S4" t="n">
-        <v>33053.02</v>
+        <v>34224.45</v>
       </c>
       <c r="T4" t="n">
-        <v>-928.84</v>
+        <v>242.59</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -903,31 +903,31 @@
         <v>1.65</v>
       </c>
       <c r="L5" t="n">
-        <v>1.49</v>
+        <v>1.81</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.097</v>
+        <v>0.097</v>
       </c>
       <c r="N5" t="n">
         <v>27126</v>
       </c>
       <c r="O5" t="n">
-        <v>31928.13</v>
+        <v>23396.71</v>
       </c>
       <c r="P5" t="n">
         <v>44757.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>47572.91</v>
+        <v>42348.04</v>
       </c>
       <c r="R5" t="n">
         <v>22514.58</v>
       </c>
       <c r="S5" t="n">
-        <v>21391.85</v>
+        <v>23162.74</v>
       </c>
       <c r="T5" t="n">
-        <v>-1122.73</v>
+        <v>648.16</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -1195,31 +1195,31 @@
         <v>1.4</v>
       </c>
       <c r="L9" t="n">
-        <v>1.49</v>
+        <v>1.26</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0643</v>
+        <v>-0.1</v>
       </c>
       <c r="N9" t="n">
         <v>38981</v>
       </c>
       <c r="O9" t="n">
-        <v>33869.56</v>
+        <v>49440.39</v>
       </c>
       <c r="P9" t="n">
         <v>54573.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>50465.65</v>
+        <v>62294.89</v>
       </c>
       <c r="R9" t="n">
         <v>27286.7</v>
       </c>
       <c r="S9" t="n">
-        <v>26756.96</v>
+        <v>27686.62</v>
       </c>
       <c r="T9" t="n">
-        <v>-529.74</v>
+        <v>399.92</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1487,31 +1487,31 @@
         <v>1.65</v>
       </c>
       <c r="L13" t="n">
-        <v>1.49</v>
+        <v>1.81</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.097</v>
+        <v>0.097</v>
       </c>
       <c r="N13" t="n">
         <v>29715</v>
       </c>
       <c r="O13" t="n">
-        <v>32609.17</v>
+        <v>27311.8</v>
       </c>
       <c r="P13" t="n">
         <v>49029.75</v>
       </c>
       <c r="Q13" t="n">
-        <v>48587.67</v>
+        <v>49434.37</v>
       </c>
       <c r="R13" t="n">
         <v>24663.45</v>
       </c>
       <c r="S13" t="n">
-        <v>21848.15</v>
+        <v>27038.69</v>
       </c>
       <c r="T13" t="n">
-        <v>-2815.3</v>
+        <v>2375.24</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -1925,31 +1925,31 @@
         <v>2.08</v>
       </c>
       <c r="L19" t="n">
-        <v>1.99</v>
+        <v>2.28</v>
       </c>
       <c r="M19" t="n">
-        <v>-0.0433</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="N19" t="n">
         <v>29503</v>
       </c>
       <c r="O19" t="n">
-        <v>30553.27</v>
+        <v>27436.95</v>
       </c>
       <c r="P19" t="n">
         <v>61366.24</v>
       </c>
       <c r="Q19" t="n">
-        <v>60801</v>
+        <v>62556.24</v>
       </c>
       <c r="R19" t="n">
         <v>30683.12</v>
       </c>
       <c r="S19" t="n">
-        <v>29025.6</v>
+        <v>34021.81</v>
       </c>
       <c r="T19" t="n">
-        <v>-1657.52</v>
+        <v>3338.69</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -1998,31 +1998,31 @@
         <v>2.95</v>
       </c>
       <c r="L20" t="n">
-        <v>2.99</v>
+        <v>2.8</v>
       </c>
       <c r="M20" t="n">
-        <v>0.0136</v>
+        <v>-0.0508</v>
       </c>
       <c r="N20" t="n">
         <v>36581</v>
       </c>
       <c r="O20" t="n">
-        <v>35549.56</v>
+        <v>40868.13</v>
       </c>
       <c r="P20" t="n">
         <v>107913.95</v>
       </c>
       <c r="Q20" t="n">
-        <v>106293.19</v>
+        <v>114430.78</v>
       </c>
       <c r="R20" t="n">
         <v>53774.07</v>
       </c>
       <c r="S20" t="n">
-        <v>53679.84</v>
+        <v>53945.94</v>
       </c>
       <c r="T20" t="n">
-        <v>-94.23</v>
+        <v>171.87</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -2728,31 +2728,31 @@
         <v>2.08</v>
       </c>
       <c r="L30" t="n">
-        <v>1.99</v>
+        <v>2.28</v>
       </c>
       <c r="M30" t="n">
-        <v>-0.0433</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="N30" t="n">
         <v>39840</v>
       </c>
       <c r="O30" t="n">
-        <v>42639.57</v>
+        <v>34602.27</v>
       </c>
       <c r="P30" t="n">
         <v>82867.2</v>
       </c>
       <c r="Q30" t="n">
-        <v>84852.75</v>
+        <v>78893.17999999999</v>
       </c>
       <c r="R30" t="n">
         <v>41433.6</v>
       </c>
       <c r="S30" t="n">
-        <v>40507.59</v>
+        <v>42906.82</v>
       </c>
       <c r="T30" t="n">
-        <v>-926.01</v>
+        <v>1473.22</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -2947,31 +2947,31 @@
         <v>2.95</v>
       </c>
       <c r="L33" t="n">
-        <v>2.99</v>
+        <v>2.66</v>
       </c>
       <c r="M33" t="n">
-        <v>0.0136</v>
+        <v>-0.0983</v>
       </c>
       <c r="N33" t="n">
         <v>15771</v>
       </c>
       <c r="O33" t="n">
-        <v>15034.7</v>
+        <v>22771.81</v>
       </c>
       <c r="P33" t="n">
         <v>46524.45</v>
       </c>
       <c r="Q33" t="n">
-        <v>44953.74</v>
+        <v>60573.02</v>
       </c>
       <c r="R33" t="n">
         <v>23183.37</v>
       </c>
       <c r="S33" t="n">
-        <v>22702.39</v>
+        <v>26870.74</v>
       </c>
       <c r="T33" t="n">
-        <v>-480.98</v>
+        <v>3687.37</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
@@ -3093,31 +3093,31 @@
         <v>2.95</v>
       </c>
       <c r="L35" t="n">
-        <v>2.99</v>
+        <v>2.88</v>
       </c>
       <c r="M35" t="n">
-        <v>0.0136</v>
+        <v>-0.0237</v>
       </c>
       <c r="N35" t="n">
         <v>18551</v>
       </c>
       <c r="O35" t="n">
-        <v>18044.63</v>
+        <v>19489.42</v>
       </c>
       <c r="P35" t="n">
         <v>54725.45</v>
       </c>
       <c r="Q35" t="n">
-        <v>53953.43</v>
+        <v>56129.54</v>
       </c>
       <c r="R35" t="n">
         <v>27269.97</v>
       </c>
       <c r="S35" t="n">
-        <v>27247.38</v>
+        <v>27285.19</v>
       </c>
       <c r="T35" t="n">
-        <v>-22.59</v>
+        <v>15.22</v>
       </c>
       <c r="U35" t="inlineStr">
         <is>
@@ -3239,31 +3239,31 @@
         <v>2.95</v>
       </c>
       <c r="L37" t="n">
-        <v>2.99</v>
+        <v>2.66</v>
       </c>
       <c r="M37" t="n">
-        <v>0.0136</v>
+        <v>-0.0983</v>
       </c>
       <c r="N37" t="n">
         <v>19597</v>
       </c>
       <c r="O37" t="n">
-        <v>18791.24</v>
+        <v>27057.44</v>
       </c>
       <c r="P37" t="n">
         <v>57811.15</v>
       </c>
       <c r="Q37" t="n">
-        <v>56185.8</v>
+        <v>71972.78999999999</v>
       </c>
       <c r="R37" t="n">
         <v>28807.59</v>
       </c>
       <c r="S37" t="n">
-        <v>28374.77</v>
+        <v>31927.78</v>
       </c>
       <c r="T37" t="n">
-        <v>-432.82</v>
+        <v>3120.19</v>
       </c>
       <c r="U37" t="inlineStr">
         <is>
@@ -3312,35 +3312,35 @@
         <v>4.95</v>
       </c>
       <c r="L38" t="n">
-        <v>4.49</v>
+        <v>4.95</v>
       </c>
       <c r="M38" t="n">
-        <v>-0.0929</v>
+        <v>0</v>
       </c>
       <c r="N38" t="n">
         <v>28378</v>
       </c>
       <c r="O38" t="n">
-        <v>34821.08</v>
+        <v>28378</v>
       </c>
       <c r="P38" t="n">
         <v>140471.1</v>
       </c>
       <c r="Q38" t="n">
-        <v>156346.63</v>
+        <v>140471.1</v>
       </c>
       <c r="R38" t="n">
         <v>70093.66</v>
       </c>
       <c r="S38" t="n">
-        <v>69990.36</v>
+        <v>70093.66</v>
       </c>
       <c r="T38" t="n">
-        <v>-103.3</v>
+        <v>0</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Optimisation Marge (Élastique)</t>
+          <t>Maintien (Gain de Marge Défavorable)</t>
         </is>
       </c>
     </row>
@@ -3677,31 +3677,31 @@
         <v>3.95</v>
       </c>
       <c r="L43" t="n">
-        <v>3.99</v>
+        <v>3.56</v>
       </c>
       <c r="M43" t="n">
-        <v>0.0101</v>
+        <v>-0.0987</v>
       </c>
       <c r="N43" t="n">
         <v>15727</v>
       </c>
       <c r="O43" t="n">
-        <v>15166.86</v>
+        <v>22863.8</v>
       </c>
       <c r="P43" t="n">
         <v>62121.65</v>
       </c>
       <c r="Q43" t="n">
-        <v>60515.77</v>
+        <v>81395.12</v>
       </c>
       <c r="R43" t="n">
         <v>30982.19</v>
       </c>
       <c r="S43" t="n">
-        <v>30485.39</v>
+        <v>36124.8</v>
       </c>
       <c r="T43" t="n">
-        <v>-496.8</v>
+        <v>5142.61</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
@@ -3969,31 +3969,31 @@
         <v>2.55</v>
       </c>
       <c r="L47" t="n">
-        <v>2.49</v>
+        <v>2.8</v>
       </c>
       <c r="M47" t="n">
-        <v>-0.0235</v>
+        <v>0.098</v>
       </c>
       <c r="N47" t="n">
         <v>32525</v>
       </c>
       <c r="O47" t="n">
-        <v>33800.89</v>
+        <v>27962.68</v>
       </c>
       <c r="P47" t="n">
         <v>82938.75</v>
       </c>
       <c r="Q47" t="n">
-        <v>84164.21000000001</v>
+        <v>78295.52</v>
       </c>
       <c r="R47" t="n">
         <v>41632</v>
       </c>
       <c r="S47" t="n">
-        <v>41237.08</v>
+        <v>42782.91</v>
       </c>
       <c r="T47" t="n">
-        <v>-394.92</v>
+        <v>1150.91</v>
       </c>
       <c r="U47" t="inlineStr">
         <is>
@@ -4352,13 +4352,13 @@
         <v>2174918.07</v>
       </c>
       <c r="D2" t="n">
-        <v>2335043.93</v>
+        <v>2373740.71</v>
       </c>
       <c r="E2" t="n">
-        <v>160125.86</v>
+        <v>198822.64</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0736</v>
+        <v>0.0914</v>
       </c>
     </row>
     <row r="3">
@@ -4374,13 +4374,13 @@
         <v>1811967.34</v>
       </c>
       <c r="D3" t="n">
-        <v>1914692.33</v>
+        <v>1946464.1</v>
       </c>
       <c r="E3" t="n">
-        <v>102724.99</v>
+        <v>134496.76</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0567</v>
+        <v>0.0742</v>
       </c>
     </row>
     <row r="4">
@@ -4396,13 +4396,13 @@
         <v>1449089.94</v>
       </c>
       <c r="D4" t="n">
-        <v>1501367.65</v>
+        <v>1533443.72</v>
       </c>
       <c r="E4" t="n">
-        <v>52277.71</v>
+        <v>84353.78</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0361</v>
+        <v>0.0582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>